<commit_message>
Merge AI-vs-software split and validation plan into 1b
Adds an engine column (model / rules / human) to the action map: of the
87.1% automated time, AI models do 53.6% and software rules 33.5%.
1b gains a who-does-what matrix, three measures kept apart (Autonomy
Rate, success rate, human time saved), an audit-failure rule, an
actor enum that separates software from AI, and a pilot plan for
validating 76%. Workbook rebuilt and recalculated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/R1-product-thinking/ai-human-split.xlsx
+++ b/outputs/R1-product-thinking/ai-human-split.xlsx
@@ -477,7 +477,7 @@
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="52" customWidth="1" min="9" max="9"/>
-    <col width="3" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
     <col width="38" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="44" customWidth="1" min="13" max="13"/>
@@ -533,6 +533,11 @@
           <t>Why this owner</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Results</t>
@@ -583,6 +588,11 @@
       <c r="I2" s="3" t="inlineStr">
         <is>
           <t>AI pre-fills from deck and website; founder confirms</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -636,6 +646,11 @@
           <t>Only the founder has the files</t>
         </is>
       </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
           <t>Count, generous (AI→H counted as AI)</t>
@@ -687,6 +702,11 @@
           <t>Document parsing</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
           <t>Time-weighted AI share</t>
@@ -738,6 +758,11 @@
           <t>Computed from extracted figures</t>
         </is>
       </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
           <t>Value-weighted AI share</t>
@@ -789,6 +814,11 @@
           <t>Rule-based rubric (A31)</t>
         </is>
       </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Manual hours / brand / month (no AI)</t>
@@ -840,6 +870,11 @@
           <t>Generated from failed rules</t>
         </is>
       </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Human hours / brand / month (with AI)</t>
@@ -891,6 +926,11 @@
           <t>Commercial judgement and reputation risk</t>
         </is>
       </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Consultant hours / month (A35, edit me)</t>
@@ -941,6 +981,11 @@
           <t>AI drafts; consultant edits and approves before anyone quotes it</t>
         </is>
       </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Brands per consultant (with AI)</t>
@@ -992,6 +1037,11 @@
           <t>Formula-driven from approved inputs</t>
         </is>
       </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Brands per consultant (no AI)</t>
@@ -1043,6 +1093,11 @@
           <t>Formula-driven</t>
         </is>
       </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Human hours per signed franchisee</t>
@@ -1094,6 +1149,25 @@
           <t>Lookup against a sourced table (A33)</t>
         </is>
       </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which AI models (time share)</t>
+        </is>
+      </c>
+      <c r="L12" s="7">
+        <f>SUMPRODUCT((J2:J38="model")*E2:E38*F2:F38*G2:G38)/SUMPRODUCT(E2:E38,F2:F38)</f>
+        <v/>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Minutes done by AI models ÷ all manual minutes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1131,6 +1205,25 @@
           <t>Rule-based v0</t>
         </is>
       </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  of which software rules (time share)</t>
+        </is>
+      </c>
+      <c r="L13" s="7">
+        <f>SUMPRODUCT((J2:J38="rules")*E2:E38*F2:F38*G2:G38)/SUMPRODUCT(E2:E38,F2:F38)</f>
+        <v/>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Minutes done by fixed rules, templates, formulas ÷ all manual minutes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1168,6 +1261,11 @@
           <t>Commercial negotiation with the founder</t>
         </is>
       </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Module</t>
@@ -1240,6 +1338,11 @@
           <t>Trust-building meeting</t>
         </is>
       </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>1 Onboarding</t>
@@ -1306,6 +1409,11 @@
           <t>Template + Model Card numbers</t>
         </is>
       </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>2 ROI Engine</t>
@@ -1372,6 +1480,11 @@
           <t>Template + Model Card numbers</t>
         </is>
       </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K17" t="inlineStr">
         <is>
           <t>3 Collateral</t>
@@ -1438,6 +1551,11 @@
           <t>Monthly creative refresh for Meta ads</t>
         </is>
       </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>4 Sales Agent</t>
@@ -1504,6 +1622,11 @@
           <t>Monthly script refresh for the agent</t>
         </is>
       </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K19" t="inlineStr">
         <is>
           <t>5 CRM</t>
@@ -1570,6 +1693,11 @@
           <t>Self-serve iterations</t>
         </is>
       </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K20" s="5" t="inlineStr">
         <is>
           <t>Total</t>
@@ -1636,6 +1764,11 @@
           <t>Brand-facing output needs a human sign-off</t>
         </is>
       </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1673,6 +1806,11 @@
           <t>AI proposes targeting and budget; human approves spend</t>
         </is>
       </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
       <c r="K22" s="13" t="inlineStr">
         <is>
           <t>Yellow cells are estimates you can edit (A19, A20, A34, A35). Blue cells recalculate.</t>
@@ -1715,6 +1853,11 @@
           <t>Webhook ingestion</t>
         </is>
       </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1752,6 +1895,11 @@
           <t>Speed-to-lead</t>
         </is>
       </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1789,6 +1937,11 @@
           <t>Core agent job</t>
         </is>
       </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1826,6 +1979,11 @@
           <t>Grounded answers only</t>
         </is>
       </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -1863,6 +2021,11 @@
           <t>Second channel</t>
         </is>
       </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1900,6 +2063,11 @@
           <t>3 emails per lead</t>
         </is>
       </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1937,6 +2105,11 @@
           <t>Template-based</t>
         </is>
       </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -1974,6 +2147,11 @@
           <t>Rule engine (Task 3)</t>
         </is>
       </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -2011,6 +2189,11 @@
           <t>Daily roll-up</t>
         </is>
       </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -2048,6 +2231,11 @@
           <t>Event log</t>
         </is>
       </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>rules</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -2085,6 +2273,11 @@
           <t>5-bullet summary</t>
         </is>
       </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -2122,6 +2315,11 @@
           <t>The flagged moments are the high-value ones</t>
         </is>
       </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -2159,6 +2357,11 @@
           <t>Transcription + checklist</t>
         </is>
       </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2196,6 +2399,11 @@
           <t>Trust and objection handling</t>
         </is>
       </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2233,6 +2441,11 @@
           <t>The revenue event</t>
         </is>
       </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2268,6 +2481,11 @@
       <c r="I38" s="3" t="inlineStr">
         <is>
           <t>AI suggests the stage from the conversation; consultant confirms</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>model</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2316,58 +2534,70 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>A19 Volumes</t>
+          <t>Engine (column J)</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>Per brand per month: 500 leads, about 150 voice calls, 60 takeovers, 20 discovery calls, 3 signed. Illustrative, not sourced.</t>
+          <t>model = an AI model does the work (extraction, drafting, conversation, summaries).  rules = fixed software (templates, schedules, formulas, logging, rule-based scores).  human = no automation. Owner says who is accountable; engine says what kind of automation does it.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>A20 Minutes and weights</t>
+          <t>A19 Volumes</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Manual minutes and 1-5 value weights are candidate estimates, to be calibrated in the pilot.</t>
+          <t>Per brand per month: 500 leads, about 150 voice calls, 60 takeovers, 20 discovery calls, 3 signed. Illustrative, not sourced.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>A34 Set-up spread</t>
+          <t>A20 Minutes and weights</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>One-off brand set-up actions are spread over a 6-month engagement: frequency 1/6 = 0.1667 per month.</t>
+          <t>Manual minutes and 1-5 value weights are candidate estimates, to be calibrated in the pilot.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>A35 Consultant hours</t>
+          <t>A34 Set-up spread</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>160 productive hours a month (8 h x 20 working days). Editable in cell L8.</t>
+          <t>One-off brand set-up actions are spread over a 6-month engagement: frequency 1/6 = 0.1667 per month.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>A35 Consultant hours</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>160 productive hours a month (8 h x 20 working days). Editable in cell L8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>outputs/R1-product-thinking/ai-human-split.csv in the GitHub repo; the write-up is 1b-ai-human-split.md.</t>
         </is>

</xml_diff>